<commit_message>
Show integer large extents in the loom_private report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/loom_private/loom_private_v1.xlsx
+++ b/results/loom_private/loom_private_v1.xlsx
@@ -429,9 +429,9 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
@@ -490,17 +490,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>pagerank</t>
+          <t>loom-private/pagerank</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>nodes=1,048,576, nodes_log2=20, iterations=20, edges=2,097,151, gpu_schedule_levels=16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of the incoming CSR (offsets and sources), out-degrees, and level schedule from pinned host memory; score and contribution initialization; all 20 Gauss-Seidel sweeps; download of the scores to pinned host memory</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -537,17 +537,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>attention</t>
+          <t>loom-private/multisensor-attention</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>query_tokens=25,000, context_tokens=250,000, sensor_lanes=3, feature_lanes=4, statistics=4, input_variant=0, audio_input_elements=75,000, imu_input_elements=750,000, score_pairs=6,250,000,000, output_elements=100,000</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload audio [Q][3] and IMU [C][3] float32 from pinned host memory; audio and IMU projections; streaming attention; residual and statistics; download output [Q][4] and the 4 statistics (the legacy loom_msa transfer-inclusive convention)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -783,9 +783,9 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
@@ -844,17 +844,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>pagerank</t>
+          <t>loom-private/pagerank</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>nodes=1,048,576, nodes_log2=20, iterations=20, edges=2,097,151, gpu_schedule_levels=16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of the incoming CSR (offsets and sources), out-degrees, and level schedule from pinned host memory; score and contribution initialization; all 20 Gauss-Seidel sweeps; download of the scores to pinned host memory</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -891,17 +891,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>attention</t>
+          <t>loom-private/multisensor-attention</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>query_tokens=25,000, context_tokens=250,000, sensor_lanes=3, feature_lanes=4, statistics=4, input_variant=0, audio_input_elements=75,000, imu_input_elements=750,000, score_pairs=6,250,000,000, output_elements=100,000</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload audio [Q][3] and IMU [C][3] float32 from pinned host memory; audio and IMU projections; streaming attention; residual and statistics; download output [Q][4] and the 4 statistics (the legacy loom_msa transfer-inclusive convention)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1137,9 +1137,9 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
@@ -1198,17 +1198,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>pagerank</t>
+          <t>loom-private/pagerank</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>nodes=1,048,576, nodes_log2=20, iterations=20, edges=2,097,151, gpu_schedule_levels=16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of the incoming CSR (offsets and sources), out-degrees, and level schedule from pinned host memory; score and contribution initialization; all 20 Gauss-Seidel sweeps; download of the scores to pinned host memory</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1245,17 +1245,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>attention</t>
+          <t>loom-private/multisensor-attention</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>query_tokens=25,000, context_tokens=250,000, sensor_lanes=3, feature_lanes=4, statistics=4, input_variant=0, audio_input_elements=75,000, imu_input_elements=750,000, score_pairs=6,250,000,000, output_elements=100,000</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload audio [Q][3] and IMU [C][3] float32 from pinned host memory; audio and IMU projections; streaming attention; residual and statistics; download output [Q][4] and the 4 statistics (the legacy loom_msa transfer-inclusive convention)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1492,8 +1492,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pagerank</t>
+          <t>loom-private/pagerank</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>c6d38a8f418469dc6581efaf287d5898563d001182685883dbb4a9ccd3b463cb</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1593,12 +1593,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>attention</t>
+          <t>loom-private/multisensor-attention</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>97c0a8fcb0644629217fba69512cf41ca05efcd05fc67754b59bdea8ae52526d</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pagerank</t>
+          <t>loom-private/pagerank</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>c6d38a8f418469dc6581efaf287d5898563d001182685883dbb4a9ccd3b463cb</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1845,12 +1845,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>attention</t>
+          <t>loom-private/multisensor-attention</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>97c0a8fcb0644629217fba69512cf41ca05efcd05fc67754b59bdea8ae52526d</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2055,12 +2055,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pagerank</t>
+          <t>loom-private/pagerank</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>c6d38a8f418469dc6581efaf287d5898563d001182685883dbb4a9ccd3b463cb</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2097,12 +2097,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>attention</t>
+          <t>loom-private/multisensor-attention</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>97c0a8fcb0644629217fba69512cf41ca05efcd05fc67754b59bdea8ae52526d</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2313,11 +2313,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2350,7 +2350,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>pagerank</t>
+          <t>loom-private/pagerank</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2360,24 +2360,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>c6d38a8f418469dc6581efaf287d5898563d001182685883dbb4a9ccd3b463cb</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>4a75f8d743ef7fe755822bab0ea0fb78009c145b</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>attention</t>
+          <t>loom-private/multisensor-attention</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2387,17 +2387,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>97c0a8fcb0644629217fba69512cf41ca05efcd05fc67754b59bdea8ae52526d</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>4a75f8d743ef7fe755822bab0ea0fb78009c145b</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Upstream uses one token count for both the audio queries and the IMU context; this workload generalizes the same generator and computation to separate query and context extents (25,000 queries attending over 250,000 context tokens). With equal extents it is the upstream computation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate the loom_private v1 report with all six contracts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/loom_private/loom_private_v1.xlsx
+++ b/results/loom_private/loom_private_v1.xlsx
@@ -429,7 +429,7 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -584,17 +584,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>decoder</t>
+          <t>loom-private/llama2c-decoder</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>batch=1,024, width=16,384, vocab=8,192, steps=4, generated_tokens=4,096, classifier_macs_per_step=137,438,953,472, classifier_macs_total=549,755,813,888, model_floats=268,451,840, model_bytes=1,073,807,360</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Prompt upload (pinned H2D, batch int32), device token reset from the prompts, all steps (rmsnorm, dense classifier matmul, softmax+argmax with on-device feedback), generated-token download (pinned D2H, batch x steps int32). Weights and working buffers are resident from setup.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -631,17 +631,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>anomaly</t>
+          <t>loom-private/mlperf-tiny-anomaly-model</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>samples=104,858, sample_elements=640, dataset_samples=40, input_float32_elements=67,109,120, input_bytes=268,436,480, output_int8_bytes=67,109,120, layers=10, macs_per_sample=264,192</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload the float32 samples [samples][640] (268,436,480 bytes at large) from pinned host memory; the inference kernel for every sample; download the int8 outputs [samples][640] (67,109,120 bytes)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -678,17 +678,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>vecadd_memory</t>
+          <t>loom-private/vecadd-memory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>length=1,048,576, multiplier=2, bias=0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of lhs and rhs from pinned host memory, the element-wise add, and download of result to pinned host memory</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -725,17 +725,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vecadd_product</t>
+          <t>loom-private/vecadd-product</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>records=1,048,576, operand_bytes=64, record_input_bytes=128, input_bytes=134,217,728, output_slot_bytes=64, output_bytes=67,108,864, fixture_bytes=128, record_period=256</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of the 128-byte-per-record inputs from pinned host memory, the lane-wise byte-sum kernel over all records, and the download of the 64-byte-per-record outputs to pinned host memory</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -783,7 +783,7 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -938,17 +938,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>decoder</t>
+          <t>loom-private/llama2c-decoder</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>batch=1,024, width=16,384, vocab=8,192, steps=4, generated_tokens=4,096, classifier_macs_per_step=137,438,953,472, classifier_macs_total=549,755,813,888, model_floats=268,451,840, model_bytes=1,073,807,360</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Prompt upload (pinned H2D, batch int32), device token reset from the prompts, all steps (rmsnorm, dense classifier matmul, softmax+argmax with on-device feedback), generated-token download (pinned D2H, batch x steps int32). Weights and working buffers are resident from setup.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -985,17 +985,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>anomaly</t>
+          <t>loom-private/mlperf-tiny-anomaly-model</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>samples=104,858, sample_elements=640, dataset_samples=40, input_float32_elements=67,109,120, input_bytes=268,436,480, output_int8_bytes=67,109,120, layers=10, macs_per_sample=264,192</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload the float32 samples [samples][640] (268,436,480 bytes at large) from pinned host memory; the inference kernel for every sample; download the int8 outputs [samples][640] (67,109,120 bytes)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1032,17 +1032,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>vecadd_memory</t>
+          <t>loom-private/vecadd-memory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>length=1,048,576, multiplier=2, bias=0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of lhs and rhs from pinned host memory, the element-wise add, and download of result to pinned host memory</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1079,17 +1079,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vecadd_product</t>
+          <t>loom-private/vecadd-product</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>records=1,048,576, operand_bytes=64, record_input_bytes=128, input_bytes=134,217,728, output_slot_bytes=64, output_bytes=67,108,864, fixture_bytes=128, record_period=256</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of the 128-byte-per-record inputs from pinned host memory, the lane-wise byte-sum kernel over all records, and the download of the 64-byte-per-record outputs to pinned host memory</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1137,7 +1137,7 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -1292,17 +1292,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>decoder</t>
+          <t>loom-private/llama2c-decoder</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>batch=1,024, width=16,384, vocab=8,192, steps=4, generated_tokens=4,096, classifier_macs_per_step=137,438,953,472, classifier_macs_total=549,755,813,888, model_floats=268,451,840, model_bytes=1,073,807,360</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Prompt upload (pinned H2D, batch int32), device token reset from the prompts, all steps (rmsnorm, dense classifier matmul, softmax+argmax with on-device feedback), generated-token download (pinned D2H, batch x steps int32). Weights and working buffers are resident from setup.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1339,17 +1339,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>anomaly</t>
+          <t>loom-private/mlperf-tiny-anomaly-model</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>samples=104,858, sample_elements=640, dataset_samples=40, input_float32_elements=67,109,120, input_bytes=268,436,480, output_int8_bytes=67,109,120, layers=10, macs_per_sample=264,192</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload the float32 samples [samples][640] (268,436,480 bytes at large) from pinned host memory; the inference kernel for every sample; download the int8 outputs [samples][640] (67,109,120 bytes)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1386,17 +1386,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>vecadd_memory</t>
+          <t>loom-private/vecadd-memory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>length=1,048,576, multiplier=2, bias=0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of lhs and rhs from pinned host memory, the element-wise add, and download of result to pinned host memory</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1433,17 +1433,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vecadd_product</t>
+          <t>loom-private/vecadd-product</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>contract pending</t>
+          <t>records=1,048,576, operand_bytes=64, record_input_bytes=128, input_bytes=134,217,728, output_slot_bytes=64, output_bytes=67,108,864, fixture_bytes=128, record_period=256</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>upload of the 128-byte-per-record inputs from pinned host memory, the lane-wise byte-sum kernel over all records, and the download of the 64-byte-per-record outputs to pinned host memory</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1492,7 +1492,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>97c0a8fcb0644629217fba69512cf41ca05efcd05fc67754b59bdea8ae52526d</t>
+          <t>e8f7a56bcebdd1408c2c1956027717fa2a9039da1d43cb553b390c1e16640190</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1635,12 +1635,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>decoder</t>
+          <t>loom-private/llama2c-decoder</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>847d3367d564ef22250df7f929c1871067c0ac048f92429d03a7e4f15165340d</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1677,12 +1677,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>anomaly</t>
+          <t>loom-private/mlperf-tiny-anomaly-model</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>7a3e32a8349e2d198d7a7d995cba546603594751b7dc8df3b8d9234dbb12adde</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>vecadd_memory</t>
+          <t>loom-private/vecadd-memory</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2cfa489f84dfc97ec02b7a5e2ff08e7f9f4a52b9f865f4325da027d422b21920</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1761,12 +1761,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>vecadd_product</t>
+          <t>loom-private/vecadd-product</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>d26fb78405a3ac250ae3866803b22e871a2083bf60292024cc2e2e0bd0e110ae</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>97c0a8fcb0644629217fba69512cf41ca05efcd05fc67754b59bdea8ae52526d</t>
+          <t>e8f7a56bcebdd1408c2c1956027717fa2a9039da1d43cb553b390c1e16640190</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1887,12 +1887,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>decoder</t>
+          <t>loom-private/llama2c-decoder</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>847d3367d564ef22250df7f929c1871067c0ac048f92429d03a7e4f15165340d</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1929,12 +1929,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>anomaly</t>
+          <t>loom-private/mlperf-tiny-anomaly-model</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>7a3e32a8349e2d198d7a7d995cba546603594751b7dc8df3b8d9234dbb12adde</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>vecadd_memory</t>
+          <t>loom-private/vecadd-memory</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2cfa489f84dfc97ec02b7a5e2ff08e7f9f4a52b9f865f4325da027d422b21920</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2013,12 +2013,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>vecadd_product</t>
+          <t>loom-private/vecadd-product</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>d26fb78405a3ac250ae3866803b22e871a2083bf60292024cc2e2e0bd0e110ae</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>97c0a8fcb0644629217fba69512cf41ca05efcd05fc67754b59bdea8ae52526d</t>
+          <t>e8f7a56bcebdd1408c2c1956027717fa2a9039da1d43cb553b390c1e16640190</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2139,12 +2139,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>decoder</t>
+          <t>loom-private/llama2c-decoder</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>847d3367d564ef22250df7f929c1871067c0ac048f92429d03a7e4f15165340d</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>anomaly</t>
+          <t>loom-private/mlperf-tiny-anomaly-model</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>7a3e32a8349e2d198d7a7d995cba546603594751b7dc8df3b8d9234dbb12adde</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>vecadd_memory</t>
+          <t>loom-private/vecadd-memory</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2cfa489f84dfc97ec02b7a5e2ff08e7f9f4a52b9f865f4325da027d422b21920</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2265,12 +2265,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>vecadd_product</t>
+          <t>loom-private/vecadd-product</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>d26fb78405a3ac250ae3866803b22e871a2083bf60292024cc2e2e0bd0e110ae</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2313,7 +2313,7 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>97c0a8fcb0644629217fba69512cf41ca05efcd05fc67754b59bdea8ae52526d</t>
+          <t>e8f7a56bcebdd1408c2c1956027717fa2a9039da1d43cb553b390c1e16640190</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2404,7 +2404,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>decoder</t>
+          <t>loom-private/llama2c-decoder</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2414,24 +2414,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>847d3367d564ef22250df7f929c1871067c0ac048f92429d03a7e4f15165340d</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>4a75f8d743ef7fe755822bab0ea0fb78009c145b</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Upstream decodes one sequence; this workload decodes 1,024 independent sequences at once (prompt of sequence b is b mod vocab), runs the classifier as one dense batch matmul per step, and keeps every sequence's token feedback on the GPU. Model, per-sequence arithmetic, and checks follow upstream.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>anomaly</t>
+          <t>loom-private/mlperf-tiny-anomaly-model</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2441,24 +2441,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>7a3e32a8349e2d198d7a7d995cba546603594751b7dc8df3b8d9234dbb12adde</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>4a75f8d743ef7fe755822bab0ea0fb78009c145b</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>A large CUDA extension of the upstream sample contract. Upstream runs the complete int8 ad01 model on at most the 40 samples of the pinned dataset (warmup samples followed by measured samples, in dataset order). This workload runs the same per-sample computation on 104,858 samples, where sample i is dataset sample i mod 40, and every sample is inferred on the GPU. Per-sample arithmetic is the upstream arithmetic, unchanged.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>vecadd_memory</t>
+          <t>loom-private/vecadd-memory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2468,24 +2468,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2cfa489f84dfc97ec02b7a5e2ff08e7f9f4a52b9f865f4325da027d422b21920</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>4a75f8d743ef7fe755822bab0ea0fb78009c145b</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Large size only. Upstream's default vector length is 64 and its preset lengths are 4096, 65536, and 131072; this port runs 1,048,576 elements (the element count of the legacy standalone vec_add.cu) with upstream's default multiplier 2 and bias 0. The kernel semantics are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vecadd_product</t>
+          <t>loom-private/vecadd-product</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2495,17 +2495,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>d26fb78405a3ac250ae3866803b22e871a2083bf60292024cc2e2e0bd0e110ae</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>4a75f8d743ef7fe755822bab0ea0fb78009c145b</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Batched CUDA extension of upstream's cached-operand product interface. Upstream holds one 128-byte cached input (two 64-byte operands) and writes one 64-byte output slot per measured sample, with warm-up samples rewriting slot 0; its host harness caps measured samples at 64. This workload instead runs 1,048,576 independent records, each with its own two 64-byte operands derived from the cached fixture, and one 64-byte output slot per record. Record 0 equals upstream's single sample.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record large-workload correctness on the RTX 3090 for the loom_private suite
Run 20261025-191236-mono-bf8619ed (results/record_run.py, GPU
GPU-94e819d6, driver 610.43.02, CUDA 13.3) at 7d1af47. Validation ran the
unit tests, the legacy freeze, asset verification, and a fresh build and
make test of all six applications. The measured command ran run_suite.py:
each application passed two Direct and two CUDA Graph invocations against
its CPU oracle with identical output digests.

Select each check record in results/loom_private/inputs/rtx3090.json and
regenerate the v1 report. Timings remain pending.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/loom_private/loom_private_v1.xlsx
+++ b/results/loom_private/loom_private_v1.xlsx
@@ -1498,7 +1498,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1561,27 +1561,27 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/pagerank/results/20261025-191236-mono-bf8619ed-check.json</t>
         </is>
       </c>
     </row>
@@ -1603,27 +1603,27 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/attention/results/20261025-191236-mono-bf8619ed-check.json</t>
         </is>
       </c>
     </row>
@@ -1645,27 +1645,27 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/decoder/results/20261025-191236-mono-bf8619ed-check.json</t>
         </is>
       </c>
     </row>
@@ -1687,27 +1687,27 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/anomaly/results/20261025-191236-mono-bf8619ed-check.json</t>
         </is>
       </c>
     </row>
@@ -1729,27 +1729,27 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/vecadd_memory/results/20261025-191236-mono-bf8619ed-check.json</t>
         </is>
       </c>
     </row>
@@ -1771,27 +1771,27 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/vecadd_product/results/20261025-191236-mono-bf8619ed-check.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Select RTX 3090, 4090, and 5090 loom_private v1 baselines
Point each GPU manifest at its recorded check and Direct/Graph bench runs
at source revision 296aa92, and simplify the generated results page: one
workload table, end-to-end and kernel-only timing tables across GPUs, one
correctness table, and a test-machine table built from the recorder
metadata (host, driver, CUDA release, source revision).
</commit_message>
<xml_diff>
--- a/results/loom_private/loom_private_v1.xlsx
+++ b/results/loom_private/loom_private_v1.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTX 4090" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTX 5090" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correctness" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contracts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contracts" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,8 +437,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,34 +504,26 @@
           <t>upload of the incoming CSR (offsets and sources), out-degrees, and level schedule from pinned host memory; score and contribution initialization; all 20 Gauss-Seidel sweeps; download of the scores to pinned host memory</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D2" t="n">
+        <v>5342.78069</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5059.07059</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4225.42877</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3923.45428</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/pagerank/results/20261025-235210-mono-afce3380-bench-direct.json</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/pagerank/results/20261025-235325-mono-34308366-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -550,34 +543,26 @@
           <t>upload audio [Q][3] and IMU [C][3] float32 from pinned host memory; audio and IMU projections; streaming attention; residual and statistics; download output [Q][4] and the 4 statistics (the legacy loom_msa transfer-inclusive convention)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D3" t="n">
+        <v>32482.9285</v>
+      </c>
+      <c r="E3" t="n">
+        <v>31979.1901</v>
+      </c>
+      <c r="F3" t="n">
+        <v>32258.7067</v>
+      </c>
+      <c r="G3" t="n">
+        <v>31877.121</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/attention/results/20261025-235210-mono-afce3380-bench-direct.json</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/attention/results/20261025-235325-mono-34308366-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -597,34 +582,26 @@
           <t>Prompt upload (pinned H2D, batch int32), device token reset from the prompts, all steps (rmsnorm, dense classifier matmul, softmax+argmax with on-device feedback), generated-token download (pinned D2H, batch x steps int32). Weights and working buffers are resident from setup.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D4" t="n">
+        <v>147572.778</v>
+      </c>
+      <c r="E4" t="n">
+        <v>149914.465</v>
+      </c>
+      <c r="F4" t="n">
+        <v>148385.437</v>
+      </c>
+      <c r="G4" t="n">
+        <v>150281.262</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/decoder/results/20261025-235210-mono-afce3380-bench-direct.json</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/decoder/results/20261025-235325-mono-34308366-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -644,34 +621,26 @@
           <t>upload the float32 samples [samples][640] (268,436,480 bytes at large) from pinned host memory; the inference kernel for every sample; download the int8 outputs [samples][640] (67,109,120 bytes)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D5" t="n">
+        <v>504419.043</v>
+      </c>
+      <c r="E5" t="n">
+        <v>511873.633</v>
+      </c>
+      <c r="F5" t="n">
+        <v>494544.336</v>
+      </c>
+      <c r="G5" t="n">
+        <v>498307.52</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/anomaly/results/20261025-235210-mono-afce3380-bench-direct.json</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/anomaly/results/20261025-235325-mono-34308366-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -691,34 +660,26 @@
           <t>upload of lhs and rhs from pinned host memory, the element-wise add, and download of result to pinned host memory</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D6" t="n">
+        <v>535.801601</v>
+      </c>
+      <c r="E6" t="n">
+        <v>534.448004</v>
+      </c>
+      <c r="F6" t="n">
+        <v>16.2816003</v>
+      </c>
+      <c r="G6" t="n">
+        <v>15.9743994</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/vecadd_memory/results/20261025-235210-mono-afce3380-bench-direct.json</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/vecadd_memory/results/20261025-235325-mono-34308366-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -738,34 +699,26 @@
           <t>upload of the 128-byte-per-record inputs from pinned host memory, the lane-wise byte-sum kernel over all records, and the download of the 64-byte-per-record outputs to pinned host memory</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D7" t="n">
+        <v>8299.51859</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8299.626920000001</v>
+      </c>
+      <c r="F7" t="n">
+        <v>237.9776</v>
+      </c>
+      <c r="G7" t="n">
+        <v>237.107205</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/vecadd_product/results/20261025-235210-mono-afce3380-bench-direct.json</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx3090/loom_private/vecadd_product/results/20261025-235325-mono-34308366-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -790,8 +743,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -857,34 +810,26 @@
           <t>upload of the incoming CSR (offsets and sources), out-degrees, and level schedule from pinned host memory; score and contribution initialization; all 20 Gauss-Seidel sweeps; download of the scores to pinned host memory</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D2" t="n">
+        <v>2483.18081</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2274.33758</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1468.5008</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1262.95042</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/pagerank/results/20261025-235536-octacos-eccbe1ac-bench-direct.json</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/pagerank/results/20261025-235634-octacos-19c4c2a0-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -904,34 +849,26 @@
           <t>upload audio [Q][3] and IMU [C][3] float32 from pinned host memory; audio and IMU projections; streaming attention; residual and statistics; download output [Q][4] and the 4 statistics (the legacy loom_msa transfer-inclusive convention)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D3" t="n">
+        <v>13231.6086</v>
+      </c>
+      <c r="E3" t="n">
+        <v>13429.5898</v>
+      </c>
+      <c r="F3" t="n">
+        <v>13969.3054</v>
+      </c>
+      <c r="G3" t="n">
+        <v>13123.0713</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/attention/results/20261025-235536-octacos-eccbe1ac-bench-direct.json</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/attention/results/20261025-235634-octacos-19c4c2a0-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -951,34 +888,26 @@
           <t>Prompt upload (pinned H2D, batch int32), device token reset from the prompts, all steps (rmsnorm, dense classifier matmul, softmax+argmax with on-device feedback), generated-token download (pinned D2H, batch x steps int32). Weights and working buffers are resident from setup.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D4" t="n">
+        <v>68298.1995</v>
+      </c>
+      <c r="E4" t="n">
+        <v>68319.8364</v>
+      </c>
+      <c r="F4" t="n">
+        <v>68762.52439999999</v>
+      </c>
+      <c r="G4" t="n">
+        <v>68812.4939</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/decoder/results/20261025-235536-octacos-eccbe1ac-bench-direct.json</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/decoder/results/20261025-235634-octacos-19c4c2a0-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -998,34 +927,26 @@
           <t>upload the float32 samples [samples][640] (268,436,480 bytes at large) from pinned host memory; the inference kernel for every sample; download the int8 outputs [samples][640] (67,109,120 bytes)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D5" t="n">
+        <v>239661.45</v>
+      </c>
+      <c r="E5" t="n">
+        <v>239624.829</v>
+      </c>
+      <c r="F5" t="n">
+        <v>226299.585</v>
+      </c>
+      <c r="G5" t="n">
+        <v>226292.114</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/anomaly/results/20261025-235536-octacos-eccbe1ac-bench-direct.json</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/anomaly/results/20261025-235634-octacos-19c4c2a0-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1045,34 +966,26 @@
           <t>upload of lhs and rhs from pinned host memory, the element-wise add, and download of result to pinned host memory</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D6" t="n">
+        <v>513.817596</v>
+      </c>
+      <c r="E6" t="n">
+        <v>512.708807</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3.94239984</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3.73760015</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/vecadd_memory/results/20261025-235536-octacos-eccbe1ac-bench-direct.json</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/vecadd_memory/results/20261025-235634-octacos-19c4c2a0-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1092,34 +1005,26 @@
           <t>upload of the 128-byte-per-record inputs from pinned host memory, the lane-wise byte-sum kernel over all records, and the download of the 64-byte-per-record outputs to pinned host memory</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D7" t="n">
+        <v>8213.64136</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8199.22867</v>
+      </c>
+      <c r="F7" t="n">
+        <v>212.531209</v>
+      </c>
+      <c r="G7" t="n">
+        <v>211.747193</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/vecadd_product/results/20261025-235536-octacos-eccbe1ac-bench-direct.json</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/vecadd_product/results/20261025-235634-octacos-19c4c2a0-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1144,8 +1049,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1211,34 +1116,26 @@
           <t>upload of the incoming CSR (offsets and sources), out-degrees, and level schedule from pinned host memory; score and contribution initialization; all 20 Gauss-Seidel sweeps; download of the scores to pinned host memory</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D2" t="n">
+        <v>1698.75526</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1569.01598</v>
+      </c>
+      <c r="F2" t="n">
+        <v>961.7199900000001</v>
+      </c>
+      <c r="G2" t="n">
+        <v>920.910358</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/pagerank/results/20261025-235302-kilia-84e59307-bench-direct.json</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/pagerank/results/20261025-235338-kilia-a3d8f65a-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1258,34 +1155,26 @@
           <t>upload audio [Q][3] and IMU [C][3] float32 from pinned host memory; audio and IMU projections; streaming attention; residual and statistics; download output [Q][4] and the 4 statistics (the legacy loom_msa transfer-inclusive convention)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D3" t="n">
+        <v>26492.395</v>
+      </c>
+      <c r="E3" t="n">
+        <v>26682.6569</v>
+      </c>
+      <c r="F3" t="n">
+        <v>26382.0923</v>
+      </c>
+      <c r="G3" t="n">
+        <v>26475.4303</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/attention/results/20261025-235302-kilia-84e59307-bench-direct.json</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/attention/results/20261025-235338-kilia-a3d8f65a-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1305,34 +1194,26 @@
           <t>Prompt upload (pinned H2D, batch int32), device token reset from the prompts, all steps (rmsnorm, dense classifier matmul, softmax+argmax with on-device feedback), generated-token download (pinned D2H, batch x steps int32). Weights and working buffers are resident from setup.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D4" t="n">
+        <v>52141.1316</v>
+      </c>
+      <c r="E4" t="n">
+        <v>52354.0527</v>
+      </c>
+      <c r="F4" t="n">
+        <v>52335.9253</v>
+      </c>
+      <c r="G4" t="n">
+        <v>52449.8352</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/decoder/results/20261025-235302-kilia-84e59307-bench-direct.json</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/decoder/results/20261025-235338-kilia-a3d8f65a-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1352,34 +1233,26 @@
           <t>upload the float32 samples [samples][640] (268,436,480 bytes at large) from pinned host memory; the inference kernel for every sample; download the int8 outputs [samples][640] (67,109,120 bytes)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D5" t="n">
+        <v>170771.228</v>
+      </c>
+      <c r="E5" t="n">
+        <v>170855.786</v>
+      </c>
+      <c r="F5" t="n">
+        <v>163177.429</v>
+      </c>
+      <c r="G5" t="n">
+        <v>163140.674</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/anomaly/results/20261025-235302-kilia-84e59307-bench-direct.json</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/anomaly/results/20261025-235338-kilia-a3d8f65a-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1399,34 +1272,26 @@
           <t>upload of lhs and rhs from pinned host memory, the element-wise add, and download of result to pinned host memory</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D6" t="n">
+        <v>401.252794</v>
+      </c>
+      <c r="E6" t="n">
+        <v>423.184013</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.87839994</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.13599983</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/vecadd_memory/results/20261025-235302-kilia-84e59307-bench-direct.json</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/vecadd_memory/results/20261025-235338-kilia-a3d8f65a-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1446,34 +1311,26 @@
           <t>upload of the 128-byte-per-record inputs from pinned host memory, the lane-wise byte-sum kernel over all records, and the download of the 64-byte-per-record outputs to pinned host memory</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="D7" t="n">
+        <v>4749.64638</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5087.68158</v>
+      </c>
+      <c r="F7" t="n">
+        <v>117.556798</v>
+      </c>
+      <c r="G7" t="n">
+        <v>117.615998</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/vecadd_product/results/20261025-235302-kilia-84e59307-bench-direct.json</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/vecadd_product/results/20261025-235338-kilia-a3d8f65a-bench-graph.json</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1438,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rtx3090/loom_private/pagerank/results/20261025-191236-mono-bf8619ed-check.json</t>
+          <t>rtx3090/loom_private/pagerank/results/20261025-234934-mono-39816759-check.json</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1480,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>rtx3090/loom_private/attention/results/20261025-191236-mono-bf8619ed-check.json</t>
+          <t>rtx3090/loom_private/attention/results/20261025-234934-mono-39816759-check.json</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1522,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>rtx3090/loom_private/decoder/results/20261025-191236-mono-bf8619ed-check.json</t>
+          <t>rtx3090/loom_private/decoder/results/20261025-234934-mono-39816759-check.json</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1564,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rtx3090/loom_private/anomaly/results/20261025-191236-mono-bf8619ed-check.json</t>
+          <t>rtx3090/loom_private/anomaly/results/20261025-234934-mono-39816759-check.json</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1606,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>rtx3090/loom_private/vecadd_memory/results/20261025-191236-mono-bf8619ed-check.json</t>
+          <t>rtx3090/loom_private/vecadd_memory/results/20261025-234934-mono-39816759-check.json</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1648,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>rtx3090/loom_private/vecadd_product/results/20261025-191236-mono-bf8619ed-check.json</t>
+          <t>rtx3090/loom_private/vecadd_product/results/20261025-234934-mono-39816759-check.json</t>
         </is>
       </c>
     </row>
@@ -1813,27 +1670,27 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/pagerank/results/20261025-235039-octacos-c1f83c8f-check.json</t>
         </is>
       </c>
     </row>
@@ -1855,27 +1712,27 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/attention/results/20261025-235039-octacos-c1f83c8f-check.json</t>
         </is>
       </c>
     </row>
@@ -1897,27 +1754,27 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/decoder/results/20261025-235039-octacos-c1f83c8f-check.json</t>
         </is>
       </c>
     </row>
@@ -1939,27 +1796,27 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/anomaly/results/20261025-235039-octacos-c1f83c8f-check.json</t>
         </is>
       </c>
     </row>
@@ -1981,27 +1838,27 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/vecadd_memory/results/20261025-235039-octacos-c1f83c8f-check.json</t>
         </is>
       </c>
     </row>
@@ -2023,27 +1880,27 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx4090/loom_private/vecadd_product/results/20261025-235039-octacos-c1f83c8f-check.json</t>
         </is>
       </c>
     </row>
@@ -2065,27 +1922,27 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/pagerank/results/20261025-235201-kilia-b66c6f3a-check.json</t>
         </is>
       </c>
     </row>
@@ -2107,27 +1964,27 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/attention/results/20261025-235201-kilia-b66c6f3a-check.json</t>
         </is>
       </c>
     </row>
@@ -2149,27 +2006,27 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/decoder/results/20261025-235201-kilia-b66c6f3a-check.json</t>
         </is>
       </c>
     </row>
@@ -2191,27 +2048,27 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/anomaly/results/20261025-235201-kilia-b66c6f3a-check.json</t>
         </is>
       </c>
     </row>
@@ -2233,27 +2090,27 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/vecadd_memory/results/20261025-235201-kilia-b66c6f3a-check.json</t>
         </is>
       </c>
     </row>
@@ -2275,27 +2132,27 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>2/2 pass</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>rtx5090/loom_private/vecadd_product/results/20261025-235201-kilia-b66c6f3a-check.json</t>
         </is>
       </c>
     </row>
@@ -2305,6 +2162,135 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Source revision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RTX 3090 (sm_86, 24 GB)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>mono</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>610.43.02</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CUDA 13.3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>296aa92</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>octacos</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>555.58.02</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CUDA 12.8</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>296aa92</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RTX 5090 (sm_120, 32 GB)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>kilia</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>615.71.10</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CUDA 13.4</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>296aa92</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Profile exactly one end-to-end invocation and tighten the report inputs
The binaries gain --action profile: one warmup invocation, then one between
cudaProfilerStart and cudaProfilerStop, which profile.py captures with nsys and
ncu capture ranges. Chunked variants launch kernels per chunk end to end but
once per kernel-only invocation, so the old instance-count rule misattributed
their kernels as setup.

The report now requires a passing check of the same variant for every bench
selection, rejects repeated or inconsistent repetitions and profiles from
another GPU, links every median to the run that holds it, counts runs per
version, and parses templated kernel names. An exported VARIANT no longer
leaks into common.mk.
</commit_message>
<xml_diff>
--- a/results/loom_private/loom_private_v1.xlsx
+++ b/results/loom_private/loom_private_v1.xlsx
@@ -5768,7 +5768,7 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -5860,7 +5860,7 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5906,7 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -5998,7 +5998,7 @@
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6044,7 +6044,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6090,7 +6090,7 @@
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6136,7 @@
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6228,7 +6228,7 @@
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6484,7 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6531,7 +6531,7 @@
       </c>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6574,7 +6574,7 @@
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6621,7 +6621,7 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6668,7 +6668,7 @@
       </c>
       <c r="I9" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="I10" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6805,7 +6805,7 @@
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6895,7 +6895,7 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6942,7 +6942,7 @@
       </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -6985,7 +6985,7 @@
       </c>
       <c r="I16" s="19" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7079,7 +7079,7 @@
       </c>
       <c r="I18" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7169,7 +7169,7 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="I21" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7259,7 +7259,7 @@
       </c>
       <c r="I22" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7306,7 +7306,7 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7353,7 +7353,7 @@
       </c>
       <c r="I24" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7396,7 +7396,7 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7443,7 +7443,7 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7490,7 +7490,7 @@
       </c>
       <c r="I27" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7533,7 @@
       </c>
       <c r="I28" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7627,7 +7627,7 @@
       </c>
       <c r="I30" s="16" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7670,7 +7670,7 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7764,7 +7764,7 @@
       </c>
       <c r="I33" s="16" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7807,7 +7807,7 @@
       </c>
       <c r="I34" s="19" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7854,7 +7854,7 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7901,7 +7901,7 @@
       </c>
       <c r="I36" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7944,7 +7944,7 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -7991,7 +7991,7 @@
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8038,7 +8038,7 @@
       </c>
       <c r="I39" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="I40" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8128,7 +8128,7 @@
       </c>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8175,7 +8175,7 @@
       </c>
       <c r="I42" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8218,7 +8218,7 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8265,7 +8265,7 @@
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8312,7 +8312,7 @@
       </c>
       <c r="I45" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8355,7 +8355,7 @@
       </c>
       <c r="I46" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8402,7 +8402,7 @@
       </c>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8449,7 +8449,7 @@
       </c>
       <c r="I48" s="16" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8492,7 +8492,7 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8539,7 +8539,7 @@
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="I51" s="16" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8629,7 +8629,7 @@
       </c>
       <c r="I52" s="19" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8676,7 +8676,7 @@
       </c>
       <c r="I53" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8723,7 +8723,7 @@
       </c>
       <c r="I54" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8766,7 +8766,7 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8813,7 +8813,7 @@
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8860,7 +8860,7 @@
       </c>
       <c r="I57" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -8903,7 +8903,7 @@
       </c>
       <c r="I58" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9140,7 +9140,7 @@
       </c>
       <c r="I5" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9187,7 +9187,7 @@
       </c>
       <c r="I6" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9228,7 +9228,7 @@
       </c>
       <c r="I7" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9275,7 +9275,7 @@
       </c>
       <c r="I8" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9316,7 @@
       </c>
       <c r="I9" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9363,7 +9363,7 @@
       </c>
       <c r="I10" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9404,7 +9404,7 @@
       </c>
       <c r="I11" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9451,7 +9451,7 @@
       </c>
       <c r="I12" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9492,7 +9492,7 @@
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9539,7 +9539,7 @@
       </c>
       <c r="I14" s="19" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9627,7 +9627,7 @@
       </c>
       <c r="I16" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9668,7 +9668,7 @@
       </c>
       <c r="I17" s="16" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9715,7 +9715,7 @@
       </c>
       <c r="I18" s="19" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9756,7 +9756,7 @@
       </c>
       <c r="I19" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9803,7 +9803,7 @@
       </c>
       <c r="I20" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9844,7 +9844,7 @@
       </c>
       <c r="I21" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9891,7 +9891,7 @@
       </c>
       <c r="I22" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9932,7 +9932,7 @@
       </c>
       <c r="I23" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -9979,7 +9979,7 @@
       </c>
       <c r="I24" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10020,7 +10020,7 @@
       </c>
       <c r="I25" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10067,7 +10067,7 @@
       </c>
       <c r="I26" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10108,7 +10108,7 @@
       </c>
       <c r="I27" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="I28" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10196,7 +10196,7 @@
       </c>
       <c r="I29" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10243,7 +10243,7 @@
       </c>
       <c r="I30" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10284,7 +10284,7 @@
       </c>
       <c r="I31" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10331,7 +10331,7 @@
       </c>
       <c r="I32" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10372,7 +10372,7 @@
       </c>
       <c r="I33" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10419,7 +10419,7 @@
       </c>
       <c r="I34" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10460,7 +10460,7 @@
       </c>
       <c r="I35" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10507,7 +10507,7 @@
       </c>
       <c r="I36" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10548,7 +10548,7 @@
       </c>
       <c r="I37" s="16" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10595,7 +10595,7 @@
       </c>
       <c r="I38" s="19" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10636,7 @@
       </c>
       <c r="I39" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10683,7 +10683,7 @@
       </c>
       <c r="I40" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10724,7 +10724,7 @@
       </c>
       <c r="I41" s="16" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10771,7 +10771,7 @@
       </c>
       <c r="I42" s="19" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10812,7 +10812,7 @@
       </c>
       <c r="I43" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10859,7 +10859,7 @@
       </c>
       <c r="I44" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10900,7 +10900,7 @@
       </c>
       <c r="I45" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10947,7 +10947,7 @@
       </c>
       <c r="I46" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -10988,7 +10988,7 @@
       </c>
       <c r="I47" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -11035,7 +11035,7 @@
       </c>
       <c r="I48" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="I49" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -11123,7 +11123,7 @@
       </c>
       <c r="I50" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -11164,7 +11164,7 @@
       </c>
       <c r="I51" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="I52" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -11321,7 +11321,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Large workloads; one row per report, kernel, and launch configuration. Each report covers the setup kernels and one end-to-end invocation. Medians and min/max describe profiled launches, not application latency or total GPU utilization. Missing metrics stay blank.</t>
+          <t>Large workloads; one row per report, kernel, and launch configuration. Each report covers one end-to-end invocation, after a warmup. Medians and min/max describe profiled launches, not application latency or total GPU utilization. Missing metrics stay blank.</t>
         </is>
       </c>
     </row>
@@ -11686,7 +11686,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Large workloads; one row per report, kernel, and launch configuration. Each report covers the setup kernels and one end-to-end invocation. Medians and min/max describe profiled launches, not application latency or total GPU utilization. Missing metrics stay blank.</t>
+          <t>Large workloads; one row per report, kernel, and launch configuration. Each report covers one end-to-end invocation, after a warmup. Medians and min/max describe profiled launches, not application latency or total GPU utilization. Missing metrics stay blank.</t>
         </is>
       </c>
     </row>
@@ -12051,7 +12051,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Large workloads; one row per report, kernel, and launch configuration. Each report covers the setup kernels and one end-to-end invocation. Medians and min/max describe profiled launches, not application latency or total GPU utilization. Missing metrics stay blank.</t>
+          <t>Large workloads; one row per report, kernel, and launch configuration. Each report covers one end-to-end invocation, after a warmup. Medians and min/max describe profiled launches, not application latency or total GPU utilization. Missing metrics stay blank.</t>
         </is>
       </c>
     </row>
@@ -14712,7 +14712,7 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -14761,7 +14761,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -14810,7 +14810,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -14859,7 +14859,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -14908,7 +14908,7 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -14957,7 +14957,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15006,7 +15006,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15055,7 +15055,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15104,7 +15104,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15153,7 +15153,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15202,7 +15202,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15251,7 +15251,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15717,7 +15717,7 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15766,7 +15766,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15815,7 +15815,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15864,7 +15864,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15913,7 +15913,7 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -15962,7 +15962,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16011,7 +16011,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16109,7 +16109,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16158,7 +16158,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16207,7 +16207,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16256,7 +16256,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16490,7 +16490,7 @@
       <c r="L5" s="13" t="n"/>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16539,7 +16539,7 @@
       <c r="L6" s="16" t="n"/>
       <c r="M6" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16602,7 +16602,7 @@
       </c>
       <c r="M7" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16649,7 +16649,7 @@
       <c r="L8" s="13" t="n"/>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16698,7 +16698,7 @@
       <c r="L9" s="16" t="n"/>
       <c r="M9" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16761,7 +16761,7 @@
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16808,7 +16808,7 @@
       <c r="L11" s="13" t="n"/>
       <c r="M11" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16857,7 +16857,7 @@
       <c r="L12" s="16" t="n"/>
       <c r="M12" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16920,7 +16920,7 @@
       </c>
       <c r="M13" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -16967,7 +16967,7 @@
       <c r="L14" s="13" t="n"/>
       <c r="M14" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17016,7 +17016,7 @@
       <c r="L15" s="16" t="n"/>
       <c r="M15" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17079,7 +17079,7 @@
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17126,7 +17126,7 @@
       <c r="L17" s="13" t="n"/>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17175,7 +17175,7 @@
       <c r="L18" s="16" t="n"/>
       <c r="M18" s="16" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17238,7 +17238,7 @@
       </c>
       <c r="M19" s="19" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17285,7 +17285,7 @@
       <c r="L20" s="13" t="n"/>
       <c r="M20" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17334,7 +17334,7 @@
       <c r="L21" s="16" t="n"/>
       <c r="M21" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17397,7 +17397,7 @@
       </c>
       <c r="M22" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17444,7 +17444,7 @@
       <c r="L23" s="13" t="n"/>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17493,7 +17493,7 @@
       <c r="L24" s="16" t="n"/>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17556,7 +17556,7 @@
       </c>
       <c r="M25" s="19" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17603,7 +17603,7 @@
       <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17652,7 +17652,7 @@
       <c r="L27" s="16" t="n"/>
       <c r="M27" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17715,7 +17715,7 @@
       </c>
       <c r="M28" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17762,7 +17762,7 @@
       <c r="L29" s="13" t="n"/>
       <c r="M29" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17811,7 +17811,7 @@
       <c r="L30" s="16" t="n"/>
       <c r="M30" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17874,7 +17874,7 @@
       </c>
       <c r="M31" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17921,7 +17921,7 @@
       <c r="L32" s="13" t="n"/>
       <c r="M32" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -17970,7 +17970,7 @@
       <c r="L33" s="16" t="n"/>
       <c r="M33" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -18033,7 +18033,7 @@
       </c>
       <c r="M34" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -18080,7 +18080,7 @@
       <c r="L35" s="13" t="n"/>
       <c r="M35" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -18129,7 +18129,7 @@
       <c r="L36" s="16" t="n"/>
       <c r="M36" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -18192,7 +18192,7 @@
       </c>
       <c r="M37" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -18239,7 +18239,7 @@
       <c r="L38" s="13" t="n"/>
       <c r="M38" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -18288,7 +18288,7 @@
       <c r="L39" s="16" t="n"/>
       <c r="M39" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18351,7 @@
       </c>
       <c r="M40" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19092,7 +19092,7 @@
       <c r="L5" s="13" t="n"/>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19141,7 +19141,7 @@
       <c r="L6" s="16" t="n"/>
       <c r="M6" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19204,7 +19204,7 @@
       </c>
       <c r="M7" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19251,7 +19251,7 @@
       <c r="L8" s="13" t="n"/>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19300,7 +19300,7 @@
       <c r="L9" s="16" t="n"/>
       <c r="M9" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19363,7 +19363,7 @@
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19410,7 +19410,7 @@
       <c r="L11" s="13" t="n"/>
       <c r="M11" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19459,7 +19459,7 @@
       <c r="L12" s="16" t="n"/>
       <c r="M12" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19522,7 +19522,7 @@
       </c>
       <c r="M13" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19569,7 +19569,7 @@
       <c r="L14" s="13" t="n"/>
       <c r="M14" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19618,7 +19618,7 @@
       <c r="L15" s="16" t="n"/>
       <c r="M15" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19681,7 +19681,7 @@
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19728,7 +19728,7 @@
       <c r="L17" s="13" t="n"/>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19777,7 +19777,7 @@
       <c r="L18" s="16" t="n"/>
       <c r="M18" s="16" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19840,7 +19840,7 @@
       </c>
       <c r="M19" s="19" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19887,7 +19887,7 @@
       <c r="L20" s="13" t="n"/>
       <c r="M20" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19936,7 +19936,7 @@
       <c r="L21" s="16" t="n"/>
       <c r="M21" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -19999,7 +19999,7 @@
       </c>
       <c r="M22" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20046,7 +20046,7 @@
       <c r="L23" s="13" t="n"/>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20095,7 +20095,7 @@
       <c r="L24" s="16" t="n"/>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20158,7 +20158,7 @@
       </c>
       <c r="M25" s="19" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20205,7 +20205,7 @@
       <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20254,7 +20254,7 @@
       <c r="L27" s="16" t="n"/>
       <c r="M27" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20317,7 +20317,7 @@
       </c>
       <c r="M28" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20364,7 +20364,7 @@
       <c r="L29" s="13" t="n"/>
       <c r="M29" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20413,7 +20413,7 @@
       <c r="L30" s="16" t="n"/>
       <c r="M30" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20476,7 +20476,7 @@
       </c>
       <c r="M31" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20523,7 +20523,7 @@
       <c r="L32" s="13" t="n"/>
       <c r="M32" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20572,7 +20572,7 @@
       <c r="L33" s="16" t="n"/>
       <c r="M33" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20635,7 +20635,7 @@
       </c>
       <c r="M34" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20682,7 +20682,7 @@
       <c r="L35" s="13" t="n"/>
       <c r="M35" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20731,7 +20731,7 @@
       <c r="L36" s="16" t="n"/>
       <c r="M36" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="M37" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20841,7 +20841,7 @@
       <c r="L38" s="13" t="n"/>
       <c r="M38" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20890,7 +20890,7 @@
       <c r="L39" s="16" t="n"/>
       <c r="M39" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -20953,7 +20953,7 @@
       </c>
       <c r="M40" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -21732,7 +21732,7 @@
       <c r="L5" s="13" t="n"/>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -21781,7 +21781,7 @@
       <c r="L6" s="16" t="n"/>
       <c r="M6" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -21844,7 +21844,7 @@
       </c>
       <c r="M7" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -21891,7 +21891,7 @@
       <c r="L8" s="13" t="n"/>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -21940,7 +21940,7 @@
       <c r="L9" s="16" t="n"/>
       <c r="M9" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22003,7 +22003,7 @@
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22050,7 +22050,7 @@
       <c r="L11" s="13" t="n"/>
       <c r="M11" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22099,7 +22099,7 @@
       <c r="L12" s="16" t="n"/>
       <c r="M12" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22162,7 +22162,7 @@
       </c>
       <c r="M13" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22209,7 +22209,7 @@
       <c r="L14" s="13" t="n"/>
       <c r="M14" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22258,7 +22258,7 @@
       <c r="L15" s="16" t="n"/>
       <c r="M15" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22321,7 +22321,7 @@
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22368,7 +22368,7 @@
       <c r="L17" s="13" t="n"/>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22417,7 +22417,7 @@
       <c r="L18" s="16" t="n"/>
       <c r="M18" s="16" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22480,7 +22480,7 @@
       </c>
       <c r="M19" s="19" t="inlineStr">
         <is>
-          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Weights stay on the GPU; copies prompts in and tokens out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22527,7 +22527,7 @@
       <c r="L20" s="13" t="n"/>
       <c r="M20" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22576,7 +22576,7 @@
       <c r="L21" s="16" t="n"/>
       <c r="M21" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22639,7 +22639,7 @@
       </c>
       <c r="M22" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22686,7 +22686,7 @@
       <c r="L23" s="13" t="n"/>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22735,7 +22735,7 @@
       <c r="L24" s="16" t="n"/>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22798,7 +22798,7 @@
       </c>
       <c r="M25" s="19" t="inlineStr">
         <is>
-          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Model loaded before timing; copies samples in and outputs out. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22845,7 +22845,7 @@
       <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22894,7 +22894,7 @@
       <c r="L27" s="16" t="n"/>
       <c r="M27" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -22957,7 +22957,7 @@
       </c>
       <c r="M28" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23004,7 +23004,7 @@
       <c r="L29" s="13" t="n"/>
       <c r="M29" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23053,7 +23053,7 @@
       <c r="L30" s="16" t="n"/>
       <c r="M30" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23116,7 +23116,7 @@
       </c>
       <c r="M31" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23163,7 +23163,7 @@
       <c r="L32" s="13" t="n"/>
       <c r="M32" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23212,7 +23212,7 @@
       <c r="L33" s="16" t="n"/>
       <c r="M33" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23275,7 +23275,7 @@
       </c>
       <c r="M34" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23322,7 +23322,7 @@
       <c r="L35" s="13" t="n"/>
       <c r="M35" s="13" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23371,7 +23371,7 @@
       <c r="L36" s="16" t="n"/>
       <c r="M36" s="16" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23434,7 +23434,7 @@
       </c>
       <c r="M37" s="19" t="inlineStr">
         <is>
-          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. Median of 2 runs.</t>
+          <t>Includes input upload and output download (pinned host memory). 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23481,7 +23481,7 @@
       <c r="L38" s="13" t="n"/>
       <c r="M38" s="13" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23530,7 +23530,7 @@
       <c r="L39" s="16" t="n"/>
       <c r="M39" s="16" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>
@@ -23593,7 +23593,7 @@
       </c>
       <c r="M40" s="19" t="inlineStr">
         <is>
-          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. Median of 2 runs.</t>
+          <t>Kernels only; inputs already on the GPU. 20 iterations/batch. One run each.</t>
         </is>
       </c>
     </row>

</xml_diff>